<commit_message>
CHANGED WHATSAPP TO EMAIL FOR INVITING USER DIRECTLY
</commit_message>
<xml_diff>
--- a/backend/app/assets/payroll/AROMAZEN_Salary_Upload_Template.xlsx
+++ b/backend/app/assets/payroll/AROMAZEN_Salary_Upload_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Data" sheetId="1" r:id="R1e243f8d071c4961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R0e9544b6b6924666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Data" sheetId="1" r:id="Rbab1acd67c0e4275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R64a6c5ec413045b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1080,6 +1080,9 @@
       <x:c r="AJ1" s="1" t="s">
         <x:v>35</x:v>
       </x:c>
+      <x:c r="AK1" t="str">
+        <x:v>Account Number</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
@@ -1170,16 +1173,1527 @@
       <x:c r="AD2" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="AE2"/>
-      <x:c r="AF2"/>
-      <x:c r="AG2"/>
-      <x:c r="AH2"/>
+      <x:c r="AE2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="AF2" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="AG2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AH2" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="AI2" t="s">
         <x:v>40</x:v>
       </x:c>
       <x:c r="AJ2" t="s">
         <x:v>40</x:v>
       </x:c>
+      <x:c r="AK2" t="str">
+        <x:v>123456789012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="AK3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="AK4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="AK5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="AK6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="AK7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="AK8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="AK9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="AK10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="AK11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="AK12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="AK13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="AK14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="AK15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="AK16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="AK17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="AK18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="AK19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="AK20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="AK21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="AK22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="AK23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="AK24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="AK25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="AK26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="AK27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="AK28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="AK29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="AK30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="AK31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="AK32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="AK33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="AK34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="AK35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="AK36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="AK37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="AK38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="AK39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="AK40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="AK41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="AK42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="AK43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="AK44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="AK45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="AK46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="AK47"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="AK48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="AK49"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="AK50"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="AK51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="AK52"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="AK53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="AK54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="AK55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="AK56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="AK57"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="AK58"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="AK59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="AK60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="AK61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="AK62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="AK63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="AK64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="AK65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="AK66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="AK67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="AK68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="AK69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="AK70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="AK71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="AK72"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="AK73"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="AK74"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="AK75"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="AK76"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="AK77"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="AK78"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="AK79"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="AK80"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="AK81"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="AK82"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="AK83"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="AK84"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="AK85"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="AK86"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="AK87"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="AK88"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="AK89"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="AK90"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="AK91"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="AK92"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="AK93"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="AK94"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="AK95"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="AK96"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="AK97"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="AK98"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="AK99"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="AK100"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="AK101"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="AK102"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="AK103"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="AK104"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="AK105"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="AK106"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="AK107"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="AK108"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="AK109"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="AK110"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="AK111"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="AK112"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="AK113"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="AK114"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="AK115"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="AK116"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="AK117"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="AK118"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="AK119"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="AK120"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="AK121"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="AK122"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="AK123"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="AK124"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="AK125"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="AK126"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="AK127"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="AK128"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="AK129"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="AK130"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="AK131"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="AK132"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="AK133"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="AK134"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="AK135"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="AK136"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="AK137"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="AK138"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="AK139"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="AK140"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="AK141"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="AK142"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="AK143"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="AK144"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="AK145"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="AK146"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="AK147"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="AK148"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="AK149"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="AK150"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="AK151"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="AK152"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="AK153"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="AK154"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="AK155"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="AK156"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="AK157"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="AK158"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="AK159"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="AK160"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="AK161"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="AK162"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="AK163"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="AK164"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="AK165"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="AK166"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="AK167"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="AK168"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="AK169"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="AK170"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="AK171"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="AK172"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="AK173"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="AK174"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="AK175"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="AK176"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="AK177"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="AK178"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="AK179"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="AK180"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="AK181"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="AK182"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="AK183"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="AK184"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="AK185"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="AK186"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="AK187"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="AK188"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="AK189"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="AK190"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="AK191"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="AK192"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="AK193"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="AK194"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="AK195"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="AK196"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="AK197"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="AK198"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="AK199"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="AK200"/>
+    </x:row>
+    <x:row r="201">
+      <x:c r="AK201"/>
+    </x:row>
+    <x:row r="202">
+      <x:c r="AK202"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="AK203"/>
+    </x:row>
+    <x:row r="204">
+      <x:c r="AK204"/>
+    </x:row>
+    <x:row r="205">
+      <x:c r="AK205"/>
+    </x:row>
+    <x:row r="206">
+      <x:c r="AK206"/>
+    </x:row>
+    <x:row r="207">
+      <x:c r="AK207"/>
+    </x:row>
+    <x:row r="208">
+      <x:c r="AK208"/>
+    </x:row>
+    <x:row r="209">
+      <x:c r="AK209"/>
+    </x:row>
+    <x:row r="210">
+      <x:c r="AK210"/>
+    </x:row>
+    <x:row r="211">
+      <x:c r="AK211"/>
+    </x:row>
+    <x:row r="212">
+      <x:c r="AK212"/>
+    </x:row>
+    <x:row r="213">
+      <x:c r="AK213"/>
+    </x:row>
+    <x:row r="214">
+      <x:c r="AK214"/>
+    </x:row>
+    <x:row r="215">
+      <x:c r="AK215"/>
+    </x:row>
+    <x:row r="216">
+      <x:c r="AK216"/>
+    </x:row>
+    <x:row r="217">
+      <x:c r="AK217"/>
+    </x:row>
+    <x:row r="218">
+      <x:c r="AK218"/>
+    </x:row>
+    <x:row r="219">
+      <x:c r="AK219"/>
+    </x:row>
+    <x:row r="220">
+      <x:c r="AK220"/>
+    </x:row>
+    <x:row r="221">
+      <x:c r="AK221"/>
+    </x:row>
+    <x:row r="222">
+      <x:c r="AK222"/>
+    </x:row>
+    <x:row r="223">
+      <x:c r="AK223"/>
+    </x:row>
+    <x:row r="224">
+      <x:c r="AK224"/>
+    </x:row>
+    <x:row r="225">
+      <x:c r="AK225"/>
+    </x:row>
+    <x:row r="226">
+      <x:c r="AK226"/>
+    </x:row>
+    <x:row r="227">
+      <x:c r="AK227"/>
+    </x:row>
+    <x:row r="228">
+      <x:c r="AK228"/>
+    </x:row>
+    <x:row r="229">
+      <x:c r="AK229"/>
+    </x:row>
+    <x:row r="230">
+      <x:c r="AK230"/>
+    </x:row>
+    <x:row r="231">
+      <x:c r="AK231"/>
+    </x:row>
+    <x:row r="232">
+      <x:c r="AK232"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="AK233"/>
+    </x:row>
+    <x:row r="234">
+      <x:c r="AK234"/>
+    </x:row>
+    <x:row r="235">
+      <x:c r="AK235"/>
+    </x:row>
+    <x:row r="236">
+      <x:c r="AK236"/>
+    </x:row>
+    <x:row r="237">
+      <x:c r="AK237"/>
+    </x:row>
+    <x:row r="238">
+      <x:c r="AK238"/>
+    </x:row>
+    <x:row r="239">
+      <x:c r="AK239"/>
+    </x:row>
+    <x:row r="240">
+      <x:c r="AK240"/>
+    </x:row>
+    <x:row r="241">
+      <x:c r="AK241"/>
+    </x:row>
+    <x:row r="242">
+      <x:c r="AK242"/>
+    </x:row>
+    <x:row r="243">
+      <x:c r="AK243"/>
+    </x:row>
+    <x:row r="244">
+      <x:c r="AK244"/>
+    </x:row>
+    <x:row r="245">
+      <x:c r="AK245"/>
+    </x:row>
+    <x:row r="246">
+      <x:c r="AK246"/>
+    </x:row>
+    <x:row r="247">
+      <x:c r="AK247"/>
+    </x:row>
+    <x:row r="248">
+      <x:c r="AK248"/>
+    </x:row>
+    <x:row r="249">
+      <x:c r="AK249"/>
+    </x:row>
+    <x:row r="250">
+      <x:c r="AK250"/>
+    </x:row>
+    <x:row r="251">
+      <x:c r="AK251"/>
+    </x:row>
+    <x:row r="252">
+      <x:c r="AK252"/>
+    </x:row>
+    <x:row r="253">
+      <x:c r="AK253"/>
+    </x:row>
+    <x:row r="254">
+      <x:c r="AK254"/>
+    </x:row>
+    <x:row r="255">
+      <x:c r="AK255"/>
+    </x:row>
+    <x:row r="256">
+      <x:c r="AK256"/>
+    </x:row>
+    <x:row r="257">
+      <x:c r="AK257"/>
+    </x:row>
+    <x:row r="258">
+      <x:c r="AK258"/>
+    </x:row>
+    <x:row r="259">
+      <x:c r="AK259"/>
+    </x:row>
+    <x:row r="260">
+      <x:c r="AK260"/>
+    </x:row>
+    <x:row r="261">
+      <x:c r="AK261"/>
+    </x:row>
+    <x:row r="262">
+      <x:c r="AK262"/>
+    </x:row>
+    <x:row r="263">
+      <x:c r="AK263"/>
+    </x:row>
+    <x:row r="264">
+      <x:c r="AK264"/>
+    </x:row>
+    <x:row r="265">
+      <x:c r="AK265"/>
+    </x:row>
+    <x:row r="266">
+      <x:c r="AK266"/>
+    </x:row>
+    <x:row r="267">
+      <x:c r="AK267"/>
+    </x:row>
+    <x:row r="268">
+      <x:c r="AK268"/>
+    </x:row>
+    <x:row r="269">
+      <x:c r="AK269"/>
+    </x:row>
+    <x:row r="270">
+      <x:c r="AK270"/>
+    </x:row>
+    <x:row r="271">
+      <x:c r="AK271"/>
+    </x:row>
+    <x:row r="272">
+      <x:c r="AK272"/>
+    </x:row>
+    <x:row r="273">
+      <x:c r="AK273"/>
+    </x:row>
+    <x:row r="274">
+      <x:c r="AK274"/>
+    </x:row>
+    <x:row r="275">
+      <x:c r="AK275"/>
+    </x:row>
+    <x:row r="276">
+      <x:c r="AK276"/>
+    </x:row>
+    <x:row r="277">
+      <x:c r="AK277"/>
+    </x:row>
+    <x:row r="278">
+      <x:c r="AK278"/>
+    </x:row>
+    <x:row r="279">
+      <x:c r="AK279"/>
+    </x:row>
+    <x:row r="280">
+      <x:c r="AK280"/>
+    </x:row>
+    <x:row r="281">
+      <x:c r="AK281"/>
+    </x:row>
+    <x:row r="282">
+      <x:c r="AK282"/>
+    </x:row>
+    <x:row r="283">
+      <x:c r="AK283"/>
+    </x:row>
+    <x:row r="284">
+      <x:c r="AK284"/>
+    </x:row>
+    <x:row r="285">
+      <x:c r="AK285"/>
+    </x:row>
+    <x:row r="286">
+      <x:c r="AK286"/>
+    </x:row>
+    <x:row r="287">
+      <x:c r="AK287"/>
+    </x:row>
+    <x:row r="288">
+      <x:c r="AK288"/>
+    </x:row>
+    <x:row r="289">
+      <x:c r="AK289"/>
+    </x:row>
+    <x:row r="290">
+      <x:c r="AK290"/>
+    </x:row>
+    <x:row r="291">
+      <x:c r="AK291"/>
+    </x:row>
+    <x:row r="292">
+      <x:c r="AK292"/>
+    </x:row>
+    <x:row r="293">
+      <x:c r="AK293"/>
+    </x:row>
+    <x:row r="294">
+      <x:c r="AK294"/>
+    </x:row>
+    <x:row r="295">
+      <x:c r="AK295"/>
+    </x:row>
+    <x:row r="296">
+      <x:c r="AK296"/>
+    </x:row>
+    <x:row r="297">
+      <x:c r="AK297"/>
+    </x:row>
+    <x:row r="298">
+      <x:c r="AK298"/>
+    </x:row>
+    <x:row r="299">
+      <x:c r="AK299"/>
+    </x:row>
+    <x:row r="300">
+      <x:c r="AK300"/>
+    </x:row>
+    <x:row r="301">
+      <x:c r="AK301"/>
+    </x:row>
+    <x:row r="302">
+      <x:c r="AK302"/>
+    </x:row>
+    <x:row r="303">
+      <x:c r="AK303"/>
+    </x:row>
+    <x:row r="304">
+      <x:c r="AK304"/>
+    </x:row>
+    <x:row r="305">
+      <x:c r="AK305"/>
+    </x:row>
+    <x:row r="306">
+      <x:c r="AK306"/>
+    </x:row>
+    <x:row r="307">
+      <x:c r="AK307"/>
+    </x:row>
+    <x:row r="308">
+      <x:c r="AK308"/>
+    </x:row>
+    <x:row r="309">
+      <x:c r="AK309"/>
+    </x:row>
+    <x:row r="310">
+      <x:c r="AK310"/>
+    </x:row>
+    <x:row r="311">
+      <x:c r="AK311"/>
+    </x:row>
+    <x:row r="312">
+      <x:c r="AK312"/>
+    </x:row>
+    <x:row r="313">
+      <x:c r="AK313"/>
+    </x:row>
+    <x:row r="314">
+      <x:c r="AK314"/>
+    </x:row>
+    <x:row r="315">
+      <x:c r="AK315"/>
+    </x:row>
+    <x:row r="316">
+      <x:c r="AK316"/>
+    </x:row>
+    <x:row r="317">
+      <x:c r="AK317"/>
+    </x:row>
+    <x:row r="318">
+      <x:c r="AK318"/>
+    </x:row>
+    <x:row r="319">
+      <x:c r="AK319"/>
+    </x:row>
+    <x:row r="320">
+      <x:c r="AK320"/>
+    </x:row>
+    <x:row r="321">
+      <x:c r="AK321"/>
+    </x:row>
+    <x:row r="322">
+      <x:c r="AK322"/>
+    </x:row>
+    <x:row r="323">
+      <x:c r="AK323"/>
+    </x:row>
+    <x:row r="324">
+      <x:c r="AK324"/>
+    </x:row>
+    <x:row r="325">
+      <x:c r="AK325"/>
+    </x:row>
+    <x:row r="326">
+      <x:c r="AK326"/>
+    </x:row>
+    <x:row r="327">
+      <x:c r="AK327"/>
+    </x:row>
+    <x:row r="328">
+      <x:c r="AK328"/>
+    </x:row>
+    <x:row r="329">
+      <x:c r="AK329"/>
+    </x:row>
+    <x:row r="330">
+      <x:c r="AK330"/>
+    </x:row>
+    <x:row r="331">
+      <x:c r="AK331"/>
+    </x:row>
+    <x:row r="332">
+      <x:c r="AK332"/>
+    </x:row>
+    <x:row r="333">
+      <x:c r="AK333"/>
+    </x:row>
+    <x:row r="334">
+      <x:c r="AK334"/>
+    </x:row>
+    <x:row r="335">
+      <x:c r="AK335"/>
+    </x:row>
+    <x:row r="336">
+      <x:c r="AK336"/>
+    </x:row>
+    <x:row r="337">
+      <x:c r="AK337"/>
+    </x:row>
+    <x:row r="338">
+      <x:c r="AK338"/>
+    </x:row>
+    <x:row r="339">
+      <x:c r="AK339"/>
+    </x:row>
+    <x:row r="340">
+      <x:c r="AK340"/>
+    </x:row>
+    <x:row r="341">
+      <x:c r="AK341"/>
+    </x:row>
+    <x:row r="342">
+      <x:c r="AK342"/>
+    </x:row>
+    <x:row r="343">
+      <x:c r="AK343"/>
+    </x:row>
+    <x:row r="344">
+      <x:c r="AK344"/>
+    </x:row>
+    <x:row r="345">
+      <x:c r="AK345"/>
+    </x:row>
+    <x:row r="346">
+      <x:c r="AK346"/>
+    </x:row>
+    <x:row r="347">
+      <x:c r="AK347"/>
+    </x:row>
+    <x:row r="348">
+      <x:c r="AK348"/>
+    </x:row>
+    <x:row r="349">
+      <x:c r="AK349"/>
+    </x:row>
+    <x:row r="350">
+      <x:c r="AK350"/>
+    </x:row>
+    <x:row r="351">
+      <x:c r="AK351"/>
+    </x:row>
+    <x:row r="352">
+      <x:c r="AK352"/>
+    </x:row>
+    <x:row r="353">
+      <x:c r="AK353"/>
+    </x:row>
+    <x:row r="354">
+      <x:c r="AK354"/>
+    </x:row>
+    <x:row r="355">
+      <x:c r="AK355"/>
+    </x:row>
+    <x:row r="356">
+      <x:c r="AK356"/>
+    </x:row>
+    <x:row r="357">
+      <x:c r="AK357"/>
+    </x:row>
+    <x:row r="358">
+      <x:c r="AK358"/>
+    </x:row>
+    <x:row r="359">
+      <x:c r="AK359"/>
+    </x:row>
+    <x:row r="360">
+      <x:c r="AK360"/>
+    </x:row>
+    <x:row r="361">
+      <x:c r="AK361"/>
+    </x:row>
+    <x:row r="362">
+      <x:c r="AK362"/>
+    </x:row>
+    <x:row r="363">
+      <x:c r="AK363"/>
+    </x:row>
+    <x:row r="364">
+      <x:c r="AK364"/>
+    </x:row>
+    <x:row r="365">
+      <x:c r="AK365"/>
+    </x:row>
+    <x:row r="366">
+      <x:c r="AK366"/>
+    </x:row>
+    <x:row r="367">
+      <x:c r="AK367"/>
+    </x:row>
+    <x:row r="368">
+      <x:c r="AK368"/>
+    </x:row>
+    <x:row r="369">
+      <x:c r="AK369"/>
+    </x:row>
+    <x:row r="370">
+      <x:c r="AK370"/>
+    </x:row>
+    <x:row r="371">
+      <x:c r="AK371"/>
+    </x:row>
+    <x:row r="372">
+      <x:c r="AK372"/>
+    </x:row>
+    <x:row r="373">
+      <x:c r="AK373"/>
+    </x:row>
+    <x:row r="374">
+      <x:c r="AK374"/>
+    </x:row>
+    <x:row r="375">
+      <x:c r="AK375"/>
+    </x:row>
+    <x:row r="376">
+      <x:c r="AK376"/>
+    </x:row>
+    <x:row r="377">
+      <x:c r="AK377"/>
+    </x:row>
+    <x:row r="378">
+      <x:c r="AK378"/>
+    </x:row>
+    <x:row r="379">
+      <x:c r="AK379"/>
+    </x:row>
+    <x:row r="380">
+      <x:c r="AK380"/>
+    </x:row>
+    <x:row r="381">
+      <x:c r="AK381"/>
+    </x:row>
+    <x:row r="382">
+      <x:c r="AK382"/>
+    </x:row>
+    <x:row r="383">
+      <x:c r="AK383"/>
+    </x:row>
+    <x:row r="384">
+      <x:c r="AK384"/>
+    </x:row>
+    <x:row r="385">
+      <x:c r="AK385"/>
+    </x:row>
+    <x:row r="386">
+      <x:c r="AK386"/>
+    </x:row>
+    <x:row r="387">
+      <x:c r="AK387"/>
+    </x:row>
+    <x:row r="388">
+      <x:c r="AK388"/>
+    </x:row>
+    <x:row r="389">
+      <x:c r="AK389"/>
+    </x:row>
+    <x:row r="390">
+      <x:c r="AK390"/>
+    </x:row>
+    <x:row r="391">
+      <x:c r="AK391"/>
+    </x:row>
+    <x:row r="392">
+      <x:c r="AK392"/>
+    </x:row>
+    <x:row r="393">
+      <x:c r="AK393"/>
+    </x:row>
+    <x:row r="394">
+      <x:c r="AK394"/>
+    </x:row>
+    <x:row r="395">
+      <x:c r="AK395"/>
+    </x:row>
+    <x:row r="396">
+      <x:c r="AK396"/>
+    </x:row>
+    <x:row r="397">
+      <x:c r="AK397"/>
+    </x:row>
+    <x:row r="398">
+      <x:c r="AK398"/>
+    </x:row>
+    <x:row r="399">
+      <x:c r="AK399"/>
+    </x:row>
+    <x:row r="400">
+      <x:c r="AK400"/>
+    </x:row>
+    <x:row r="401">
+      <x:c r="AK401"/>
+    </x:row>
+    <x:row r="402">
+      <x:c r="AK402"/>
+    </x:row>
+    <x:row r="403">
+      <x:c r="AK403"/>
+    </x:row>
+    <x:row r="404">
+      <x:c r="AK404"/>
+    </x:row>
+    <x:row r="405">
+      <x:c r="AK405"/>
+    </x:row>
+    <x:row r="406">
+      <x:c r="AK406"/>
+    </x:row>
+    <x:row r="407">
+      <x:c r="AK407"/>
+    </x:row>
+    <x:row r="408">
+      <x:c r="AK408"/>
+    </x:row>
+    <x:row r="409">
+      <x:c r="AK409"/>
+    </x:row>
+    <x:row r="410">
+      <x:c r="AK410"/>
+    </x:row>
+    <x:row r="411">
+      <x:c r="AK411"/>
+    </x:row>
+    <x:row r="412">
+      <x:c r="AK412"/>
+    </x:row>
+    <x:row r="413">
+      <x:c r="AK413"/>
+    </x:row>
+    <x:row r="414">
+      <x:c r="AK414"/>
+    </x:row>
+    <x:row r="415">
+      <x:c r="AK415"/>
+    </x:row>
+    <x:row r="416">
+      <x:c r="AK416"/>
+    </x:row>
+    <x:row r="417">
+      <x:c r="AK417"/>
+    </x:row>
+    <x:row r="418">
+      <x:c r="AK418"/>
+    </x:row>
+    <x:row r="419">
+      <x:c r="AK419"/>
+    </x:row>
+    <x:row r="420">
+      <x:c r="AK420"/>
+    </x:row>
+    <x:row r="421">
+      <x:c r="AK421"/>
+    </x:row>
+    <x:row r="422">
+      <x:c r="AK422"/>
+    </x:row>
+    <x:row r="423">
+      <x:c r="AK423"/>
+    </x:row>
+    <x:row r="424">
+      <x:c r="AK424"/>
+    </x:row>
+    <x:row r="425">
+      <x:c r="AK425"/>
+    </x:row>
+    <x:row r="426">
+      <x:c r="AK426"/>
+    </x:row>
+    <x:row r="427">
+      <x:c r="AK427"/>
+    </x:row>
+    <x:row r="428">
+      <x:c r="AK428"/>
+    </x:row>
+    <x:row r="429">
+      <x:c r="AK429"/>
+    </x:row>
+    <x:row r="430">
+      <x:c r="AK430"/>
+    </x:row>
+    <x:row r="431">
+      <x:c r="AK431"/>
+    </x:row>
+    <x:row r="432">
+      <x:c r="AK432"/>
+    </x:row>
+    <x:row r="433">
+      <x:c r="AK433"/>
+    </x:row>
+    <x:row r="434">
+      <x:c r="AK434"/>
+    </x:row>
+    <x:row r="435">
+      <x:c r="AK435"/>
+    </x:row>
+    <x:row r="436">
+      <x:c r="AK436"/>
+    </x:row>
+    <x:row r="437">
+      <x:c r="AK437"/>
+    </x:row>
+    <x:row r="438">
+      <x:c r="AK438"/>
+    </x:row>
+    <x:row r="439">
+      <x:c r="AK439"/>
+    </x:row>
+    <x:row r="440">
+      <x:c r="AK440"/>
+    </x:row>
+    <x:row r="441">
+      <x:c r="AK441"/>
+    </x:row>
+    <x:row r="442">
+      <x:c r="AK442"/>
+    </x:row>
+    <x:row r="443">
+      <x:c r="AK443"/>
+    </x:row>
+    <x:row r="444">
+      <x:c r="AK444"/>
+    </x:row>
+    <x:row r="445">
+      <x:c r="AK445"/>
+    </x:row>
+    <x:row r="446">
+      <x:c r="AK446"/>
+    </x:row>
+    <x:row r="447">
+      <x:c r="AK447"/>
+    </x:row>
+    <x:row r="448">
+      <x:c r="AK448"/>
+    </x:row>
+    <x:row r="449">
+      <x:c r="AK449"/>
+    </x:row>
+    <x:row r="450">
+      <x:c r="AK450"/>
+    </x:row>
+    <x:row r="451">
+      <x:c r="AK451"/>
+    </x:row>
+    <x:row r="452">
+      <x:c r="AK452"/>
+    </x:row>
+    <x:row r="453">
+      <x:c r="AK453"/>
+    </x:row>
+    <x:row r="454">
+      <x:c r="AK454"/>
+    </x:row>
+    <x:row r="455">
+      <x:c r="AK455"/>
+    </x:row>
+    <x:row r="456">
+      <x:c r="AK456"/>
+    </x:row>
+    <x:row r="457">
+      <x:c r="AK457"/>
+    </x:row>
+    <x:row r="458">
+      <x:c r="AK458"/>
+    </x:row>
+    <x:row r="459">
+      <x:c r="AK459"/>
+    </x:row>
+    <x:row r="460">
+      <x:c r="AK460"/>
+    </x:row>
+    <x:row r="461">
+      <x:c r="AK461"/>
+    </x:row>
+    <x:row r="462">
+      <x:c r="AK462"/>
+    </x:row>
+    <x:row r="463">
+      <x:c r="AK463"/>
+    </x:row>
+    <x:row r="464">
+      <x:c r="AK464"/>
+    </x:row>
+    <x:row r="465">
+      <x:c r="AK465"/>
+    </x:row>
+    <x:row r="466">
+      <x:c r="AK466"/>
+    </x:row>
+    <x:row r="467">
+      <x:c r="AK467"/>
+    </x:row>
+    <x:row r="468">
+      <x:c r="AK468"/>
+    </x:row>
+    <x:row r="469">
+      <x:c r="AK469"/>
+    </x:row>
+    <x:row r="470">
+      <x:c r="AK470"/>
+    </x:row>
+    <x:row r="471">
+      <x:c r="AK471"/>
+    </x:row>
+    <x:row r="472">
+      <x:c r="AK472"/>
+    </x:row>
+    <x:row r="473">
+      <x:c r="AK473"/>
+    </x:row>
+    <x:row r="474">
+      <x:c r="AK474"/>
+    </x:row>
+    <x:row r="475">
+      <x:c r="AK475"/>
+    </x:row>
+    <x:row r="476">
+      <x:c r="AK476"/>
+    </x:row>
+    <x:row r="477">
+      <x:c r="AK477"/>
+    </x:row>
+    <x:row r="478">
+      <x:c r="AK478"/>
+    </x:row>
+    <x:row r="479">
+      <x:c r="AK479"/>
+    </x:row>
+    <x:row r="480">
+      <x:c r="AK480"/>
+    </x:row>
+    <x:row r="481">
+      <x:c r="AK481"/>
+    </x:row>
+    <x:row r="482">
+      <x:c r="AK482"/>
+    </x:row>
+    <x:row r="483">
+      <x:c r="AK483"/>
+    </x:row>
+    <x:row r="484">
+      <x:c r="AK484"/>
+    </x:row>
+    <x:row r="485">
+      <x:c r="AK485"/>
+    </x:row>
+    <x:row r="486">
+      <x:c r="AK486"/>
+    </x:row>
+    <x:row r="487">
+      <x:c r="AK487"/>
+    </x:row>
+    <x:row r="488">
+      <x:c r="AK488"/>
+    </x:row>
+    <x:row r="489">
+      <x:c r="AK489"/>
+    </x:row>
+    <x:row r="490">
+      <x:c r="AK490"/>
+    </x:row>
+    <x:row r="491">
+      <x:c r="AK491"/>
+    </x:row>
+    <x:row r="492">
+      <x:c r="AK492"/>
+    </x:row>
+    <x:row r="493">
+      <x:c r="AK493"/>
+    </x:row>
+    <x:row r="494">
+      <x:c r="AK494"/>
+    </x:row>
+    <x:row r="495">
+      <x:c r="AK495"/>
+    </x:row>
+    <x:row r="496">
+      <x:c r="AK496"/>
+    </x:row>
+    <x:row r="497">
+      <x:c r="AK497"/>
+    </x:row>
+    <x:row r="498">
+      <x:c r="AK498"/>
+    </x:row>
+    <x:row r="499">
+      <x:c r="AK499"/>
+    </x:row>
+    <x:row r="500">
+      <x:c r="AK500"/>
+    </x:row>
+    <x:row r="501">
+      <x:c r="AK501"/>
+    </x:row>
+    <x:row r="502">
+      <x:c r="AK502"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1205,7 +2719,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Use one row per employee. Employee name, personal email, date of birth, employee code and Unit 1, 2 or 3 are mandatory. Unit Address can be left blank.</x:v>
+        <x:v>Use one row per employee. Employee name, personal email, date of birth, employee code, Unit 1, 2 or 3, Account Number, Days and Present Days are mandatory. Unit Address can be left blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>